<commit_message>
Refactor product models, enums, and seeders; update mappings
- Add partial classes and methods for Product, ProductStock, ProductPrice
- Update constructors and setters for easier instantiation
- Change InventoryType enum values to MadeToOrder, StockTracked
- Fix BranchConfiguration table name to "Branches"
- Add BranchCode to ProductStockRecord
- Change BranchRecord times from TimeOnly to TimeSpan
- Update AutoMapper profiles for new/changed properties
- Refactor seeders to resolve foreign keys by name/code with validation
- Update RestaurantData.xlsx Excel data file
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -3,13 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{803FD1A4-732F-4797-86C2-03C0D52EF12B}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BA5639D-7616-471B-ADDC-70C548AA91AA}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="5" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
     <sheet name="Brands" sheetId="2" r:id="rId2"/>
+    <sheet name="Branches" sheetId="3" r:id="rId3"/>
+    <sheet name="Products" sheetId="4" r:id="rId4"/>
+    <sheet name="ProductPrices" sheetId="5" r:id="rId5"/>
+    <sheet name="ProductStocks" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -35,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="305">
   <si>
     <t>Name</t>
   </si>
@@ -401,19 +405,573 @@
   </si>
   <si>
     <t>Japanese dairy and confectionery brand offering milk, yogurt, and chocolate products.</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>PhoneNumber</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Latitude</t>
+  </si>
+  <si>
+    <t>Longitude</t>
+  </si>
+  <si>
+    <t>OpenTime</t>
+  </si>
+  <si>
+    <t>CloseTime</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Thủ Dầu Một</t>
+  </si>
+  <si>
+    <t>BD001</t>
+  </si>
+  <si>
+    <t>bd001@store.local</t>
+  </si>
+  <si>
+    <t>123 Đại lộ Bình Dương, TP. Thủ Dầu Một, Bình Dương</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Thuận An</t>
+  </si>
+  <si>
+    <t>BD002</t>
+  </si>
+  <si>
+    <t>bd002@store.local</t>
+  </si>
+  <si>
+    <t>45 Nguyễn Văn Tiết, TP. Thuận An, Bình Dương</t>
+  </si>
+  <si>
+    <t>Dĩ An</t>
+  </si>
+  <si>
+    <t>BD003</t>
+  </si>
+  <si>
+    <t>bd003@store.local</t>
+  </si>
+  <si>
+    <t>88 Quốc lộ 1K, TP. Dĩ An, Bình Dương</t>
+  </si>
+  <si>
+    <t>Bến Cát</t>
+  </si>
+  <si>
+    <t>BD004</t>
+  </si>
+  <si>
+    <t>bd004@store.local</t>
+  </si>
+  <si>
+    <t>12 Hùng Vương, TP. Bến Cát, Bình Dương</t>
+  </si>
+  <si>
+    <t>Tân Uyên</t>
+  </si>
+  <si>
+    <t>BD005</t>
+  </si>
+  <si>
+    <t>bd005@store.local</t>
+  </si>
+  <si>
+    <t>99 DT746, TP. Tân Uyên, Bình Dương</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>InventoryType</t>
+  </si>
+  <si>
+    <t>BrandName</t>
+  </si>
+  <si>
+    <t>CategoryName</t>
+  </si>
+  <si>
+    <t>Spring Rolls</t>
+  </si>
+  <si>
+    <t>Crispy fried spring rolls served with sweet chili sauce.</t>
+  </si>
+  <si>
+    <t>MadeToOrder</t>
+  </si>
+  <si>
+    <t>Fresh Summer Rolls</t>
+  </si>
+  <si>
+    <t>Rice paper rolls with shrimp and fresh vegetables.</t>
+  </si>
+  <si>
+    <t>Garlic Bread</t>
+  </si>
+  <si>
+    <t>Toasted bread topped with garlic butter.</t>
+  </si>
+  <si>
+    <t>Grilled Beef Steak</t>
+  </si>
+  <si>
+    <t>Premium grilled beef steak with black pepper sauce.</t>
+  </si>
+  <si>
+    <t>Chicken Parmigiana</t>
+  </si>
+  <si>
+    <t>Breaded chicken topped with tomato sauce and cheese.</t>
+  </si>
+  <si>
+    <t>Crispy Fried Chicken</t>
+  </si>
+  <si>
+    <t>Golden crispy fried chicken served with fries.</t>
+  </si>
+  <si>
+    <t>Beef Fried Rice</t>
+  </si>
+  <si>
+    <t>Stir-fried rice with sliced beef and vegetables.</t>
+  </si>
+  <si>
+    <t>Seafood Fried Rice</t>
+  </si>
+  <si>
+    <t>Fried rice with shrimp, squid and mixed vegetables.</t>
+  </si>
+  <si>
+    <t>Chicken Fried Rice</t>
+  </si>
+  <si>
+    <t>Fried rice with marinated chicken.</t>
+  </si>
+  <si>
+    <t>Beef Pho</t>
+  </si>
+  <si>
+    <t>Traditional Vietnamese beef noodle soup.</t>
+  </si>
+  <si>
+    <t>Stir-fried Udon</t>
+  </si>
+  <si>
+    <t>Japanese udon noodles with beef and vegetables.</t>
+  </si>
+  <si>
+    <t>Seafood Ramen</t>
+  </si>
+  <si>
+    <t>Japanese ramen topped with assorted seafood.</t>
+  </si>
+  <si>
+    <t>Pumpkin Soup</t>
+  </si>
+  <si>
+    <t>Creamy pumpkin soup with fresh cream.</t>
+  </si>
+  <si>
+    <t>Mushroom Soup</t>
+  </si>
+  <si>
+    <t>Creamy mushroom soup served hot.</t>
+  </si>
+  <si>
+    <t>Seafood Chowder</t>
+  </si>
+  <si>
+    <t>Rich seafood soup with cream and potatoes.</t>
+  </si>
+  <si>
+    <t>Grilled Salmon</t>
+  </si>
+  <si>
+    <t>Fresh salmon grilled with lemon butter.</t>
+  </si>
+  <si>
+    <t>Garlic Butter Shrimp</t>
+  </si>
+  <si>
+    <t>Shrimp sautéed in garlic butter sauce.</t>
+  </si>
+  <si>
+    <t>Steamed Clams</t>
+  </si>
+  <si>
+    <t>Fresh clams steamed with lemongrass.</t>
+  </si>
+  <si>
+    <t>BBQ Pork Ribs</t>
+  </si>
+  <si>
+    <t>Slow-cooked barbecue pork ribs.</t>
+  </si>
+  <si>
+    <t>Grilled Chicken Skewers</t>
+  </si>
+  <si>
+    <t>Charcoal grilled chicken skewers.</t>
+  </si>
+  <si>
+    <t>Beef BBQ</t>
+  </si>
+  <si>
+    <t>Marinated beef grilled over charcoal.</t>
+  </si>
+  <si>
+    <t>Seafood Hot Pot</t>
+  </si>
+  <si>
+    <t>Mixed seafood served with rich broth.</t>
+  </si>
+  <si>
+    <t>Beef Hot Pot</t>
+  </si>
+  <si>
+    <t>Sliced beef served with vegetables and broth.</t>
+  </si>
+  <si>
+    <t>Mushroom Hot Pot</t>
+  </si>
+  <si>
+    <t>Vegetarian mushroom hot pot.</t>
+  </si>
+  <si>
+    <t>Stir-fried Vegetables</t>
+  </si>
+  <si>
+    <t>Seasonal vegetables stir-fried with garlic.</t>
+  </si>
+  <si>
+    <t>Tofu with Mushroom</t>
+  </si>
+  <si>
+    <t>Braised tofu with mixed mushrooms.</t>
+  </si>
+  <si>
+    <t>Vegan Fried Rice</t>
+  </si>
+  <si>
+    <t>Fried rice prepared without meat.</t>
+  </si>
+  <si>
+    <t>Caesar Salad</t>
+  </si>
+  <si>
+    <t>Romaine lettuce with Caesar dressing.</t>
+  </si>
+  <si>
+    <t>Tuna Salad</t>
+  </si>
+  <si>
+    <t>Fresh tuna with mixed greens.</t>
+  </si>
+  <si>
+    <t>Garden Salad</t>
+  </si>
+  <si>
+    <t>Mixed vegetables with vinaigrette dressing.</t>
+  </si>
+  <si>
+    <t>Chocolate Lava Cake</t>
+  </si>
+  <si>
+    <t>Warm chocolate cake with molten center.</t>
+  </si>
+  <si>
+    <t>Vanilla Ice Cream</t>
+  </si>
+  <si>
+    <t>Classic vanilla ice cream.</t>
+  </si>
+  <si>
+    <t>Mango Pudding</t>
+  </si>
+  <si>
+    <t>Fresh mango pudding topped with cream.</t>
+  </si>
+  <si>
+    <t>Coca-Cola Original</t>
+  </si>
+  <si>
+    <t>Carbonated soft drink.</t>
+  </si>
+  <si>
+    <t>StockTracked</t>
+  </si>
+  <si>
+    <t>Coca-Cola Zero</t>
+  </si>
+  <si>
+    <t>Sugar-free soft drink.</t>
+  </si>
+  <si>
+    <t>Refreshing cola beverage.</t>
+  </si>
+  <si>
+    <t>Pepsi Black</t>
+  </si>
+  <si>
+    <t>Zero sugar cola beverage.</t>
+  </si>
+  <si>
+    <t>Aquafina Water</t>
+  </si>
+  <si>
+    <t>Purified bottled drinking water.</t>
+  </si>
+  <si>
+    <t>Dasani Water</t>
+  </si>
+  <si>
+    <t>Purified bottled water.</t>
+  </si>
+  <si>
+    <t>Lavie Mineral Water</t>
+  </si>
+  <si>
+    <t>Natural mineral water.</t>
+  </si>
+  <si>
+    <t>Red Bull Energy Drink</t>
+  </si>
+  <si>
+    <t>Classic energy drink.</t>
+  </si>
+  <si>
+    <t>Sting Strawberry</t>
+  </si>
+  <si>
+    <t>Strawberry flavored energy drink.</t>
+  </si>
+  <si>
+    <t>Number One Energy</t>
+  </si>
+  <si>
+    <t>Energy drink with vitamins.</t>
+  </si>
+  <si>
+    <t>Milo Drink</t>
+  </si>
+  <si>
+    <t>Ready-to-drink chocolate malt beverage.</t>
+  </si>
+  <si>
+    <t>Ovaltine Drink</t>
+  </si>
+  <si>
+    <t>Chocolate malt beverage.</t>
+  </si>
+  <si>
+    <t>Vinamilk Fresh Milk</t>
+  </si>
+  <si>
+    <t>Pasteurized fresh milk.</t>
+  </si>
+  <si>
+    <t>TH true MILK Fresh Milk</t>
+  </si>
+  <si>
+    <t>Premium fresh milk.</t>
+  </si>
+  <si>
+    <t>Yakult Probiotic Drink</t>
+  </si>
+  <si>
+    <t>Fermented probiotic milk drink.</t>
+  </si>
+  <si>
+    <t>Nescafé Coffee</t>
+  </si>
+  <si>
+    <t>Instant coffee beverage.</t>
+  </si>
+  <si>
+    <t>G7 Instant Coffee</t>
+  </si>
+  <si>
+    <t>Vietnamese instant coffee.</t>
+  </si>
+  <si>
+    <t>Trung Nguyên Legend Coffee</t>
+  </si>
+  <si>
+    <t>Premium Vietnamese coffee.</t>
+  </si>
+  <si>
+    <t>Lipton Lemon Tea</t>
+  </si>
+  <si>
+    <t>Bottled lemon tea.</t>
+  </si>
+  <si>
+    <t>Fuze Tea Green Tea</t>
+  </si>
+  <si>
+    <t>Ready-to-drink green tea.</t>
+  </si>
+  <si>
+    <t>Chef Special Steak</t>
+  </si>
+  <si>
+    <t>Signature grilled steak with house sauce.</t>
+  </si>
+  <si>
+    <t>Signature Seafood Platter</t>
+  </si>
+  <si>
+    <t>Mixed premium seafood platter.</t>
+  </si>
+  <si>
+    <t>Family Combo A</t>
+  </si>
+  <si>
+    <t>Meal set for 4 people.</t>
+  </si>
+  <si>
+    <t>Family Combo B</t>
+  </si>
+  <si>
+    <t>Meal set including seafood and grilled meats.</t>
+  </si>
+  <si>
+    <t>Kids Chicken Nuggets</t>
+  </si>
+  <si>
+    <t>Chicken nuggets with fries.</t>
+  </si>
+  <si>
+    <t>Kids Spaghetti</t>
+  </si>
+  <si>
+    <t>Small portion spaghetti with tomato sauce.</t>
+  </si>
+  <si>
+    <t>American Breakfast</t>
+  </si>
+  <si>
+    <t>Eggs, bacon, toast and coffee.</t>
+  </si>
+  <si>
+    <t>Vietnamese Breakfast Combo</t>
+  </si>
+  <si>
+    <t>Beef pho with iced tea.</t>
+  </si>
+  <si>
+    <t>Lunch Combo Beef</t>
+  </si>
+  <si>
+    <t>Beef rice with soft drink.</t>
+  </si>
+  <si>
+    <t>Lunch Combo Chicken</t>
+  </si>
+  <si>
+    <t>Chicken rice with soup.</t>
+  </si>
+  <si>
+    <t>Premium Dinner Set</t>
+  </si>
+  <si>
+    <t>Three-course dinner menu.</t>
+  </si>
+  <si>
+    <t>French Fries</t>
+  </si>
+  <si>
+    <t>Crispy potato fries.</t>
+  </si>
+  <si>
+    <t>Mashed Potatoes</t>
+  </si>
+  <si>
+    <t>Creamy mashed potatoes.</t>
+  </si>
+  <si>
+    <t>Buttered Corn</t>
+  </si>
+  <si>
+    <t>Sweet corn with butter.</t>
+  </si>
+  <si>
+    <t>Summer Seafood Platter</t>
+  </si>
+  <si>
+    <t>Limited seasonal seafood selection.</t>
+  </si>
+  <si>
+    <t>Autumn Mushroom Soup</t>
+  </si>
+  <si>
+    <t>Seasonal mushroom soup.</t>
+  </si>
+  <si>
+    <t>UnitPrice</t>
+  </si>
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>QuantityOnHand</t>
+  </si>
+  <si>
+    <t>BranchCode</t>
+  </si>
+  <si>
+    <t>Can</t>
+  </si>
+  <si>
+    <t>Bottle</t>
+  </si>
+  <si>
+    <t>Box</t>
+  </si>
+  <si>
+    <t>Pack</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -436,9 +994,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1273,4 +1833,2196 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89B1122B-11C7-424E-B7BF-C058DC4DE014}">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2743888888</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F2" s="2">
+        <v>10.980460000000001</v>
+      </c>
+      <c r="G2" s="2">
+        <v>106.651856</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2743777777</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F3" s="2">
+        <v>10.911149999999999</v>
+      </c>
+      <c r="G3" s="2">
+        <v>106.71559000000001</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2743666666</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F4" s="2">
+        <v>10.903890000000001</v>
+      </c>
+      <c r="G4" s="2">
+        <v>106.76945000000001</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2743555555</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="F5" s="2">
+        <v>11.1188</v>
+      </c>
+      <c r="G5" s="2">
+        <v>106.6095</v>
+      </c>
+      <c r="H5" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2743444444</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" s="2">
+        <v>11.0525</v>
+      </c>
+      <c r="G6" s="2">
+        <v>106.7569</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C96709D-69E6-4452-AE6C-775F5C5E2849}">
+  <dimension ref="A1:E70"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80819B70-7F25-4733-9F14-1831EC4BC166}">
+  <dimension ref="A1:B70"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="27.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1">
+        <v>55000</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="1">
+        <v>65000</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="1">
+        <v>35000</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="1">
+        <v>285000</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="1">
+        <v>165000</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="1">
+        <v>145000</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1">
+        <v>89000</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="1">
+        <v>99000</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="1">
+        <v>79000</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="1">
+        <v>85000</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="1">
+        <v>115000</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="1">
+        <v>139000</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="1">
+        <v>65000</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="1">
+        <v>69000</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="1">
+        <v>109000</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="1">
+        <v>245000</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="1">
+        <v>189000</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="1">
+        <v>159000</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="1">
+        <v>279000</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1">
+        <v>149000</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="1">
+        <v>199000</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="1">
+        <v>459000</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="1">
+        <v>399000</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="1">
+        <v>329000</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="1">
+        <v>69000</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="1">
+        <v>79000</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="1">
+        <v>75000</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="1">
+        <v>85000</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="1">
+        <v>99000</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="1">
+        <v>69000</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="1">
+        <v>79000</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="1">
+        <v>45000</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="1">
+        <v>49000</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="1">
+        <v>18000</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="1">
+        <v>18000</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="1">
+        <v>18000</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="1">
+        <v>18000</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="1">
+        <v>12000</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="1">
+        <v>12000</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="1">
+        <v>10000</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="1">
+        <v>25000</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="1">
+        <v>18000</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="1">
+        <v>18000</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="1">
+        <v>22000</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="1">
+        <v>22000</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="1">
+        <v>28000</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="1">
+        <v>32000</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="1">
+        <v>15000</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="1">
+        <v>25000</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="1">
+        <v>28000</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="1">
+        <v>35000</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="1">
+        <v>22000</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="1">
+        <v>22000</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="1">
+        <v>359000</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="1">
+        <v>499000</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="1">
+        <v>799000</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="1">
+        <v>999000</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="1">
+        <v>79000</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="1">
+        <v>75000</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="1">
+        <v>119000</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="1">
+        <v>99000</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="1">
+        <v>129000</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="1">
+        <v>119000</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="1">
+        <v>499000</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="1">
+        <v>45000</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="1">
+        <v>49000</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="1">
+        <v>39000</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="1">
+        <v>599000</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="1">
+        <v>89000</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>294</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7E580B3-9B39-401F-B0BE-9E4BBC907E03}">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>298</v>
+      </c>
+      <c r="B1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1" t="s">
+        <v>297</v>
+      </c>
+      <c r="D1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B3">
+        <v>100</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>301</v>
+      </c>
+      <c r="B4">
+        <v>60</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>301</v>
+      </c>
+      <c r="B5">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>302</v>
+      </c>
+      <c r="B6">
+        <v>90</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>302</v>
+      </c>
+      <c r="B7">
+        <v>90</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>302</v>
+      </c>
+      <c r="B8">
+        <v>50</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>301</v>
+      </c>
+      <c r="B9">
+        <v>70</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>302</v>
+      </c>
+      <c r="B10">
+        <v>10</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>302</v>
+      </c>
+      <c r="B11">
+        <v>80</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>303</v>
+      </c>
+      <c r="B12">
+        <v>90</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>303</v>
+      </c>
+      <c r="B13">
+        <v>50</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>303</v>
+      </c>
+      <c r="B14">
+        <v>80</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>303</v>
+      </c>
+      <c r="B15">
+        <v>60</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>302</v>
+      </c>
+      <c r="B16">
+        <v>20</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>304</v>
+      </c>
+      <c r="B17">
+        <v>100</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>304</v>
+      </c>
+      <c r="B18">
+        <v>60</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>304</v>
+      </c>
+      <c r="B19">
+        <v>40</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>302</v>
+      </c>
+      <c r="B20">
+        <v>80</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>302</v>
+      </c>
+      <c r="B21">
+        <v>90</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor: Replace Category with ProductCategory entity
Replaced all usages of the Category entity and related logic with ProductCategory across application, domain, persistence, and API layers. Updated Product to reference ProductCategory. Removed CategoriesController and added ProductCategoriesController. Updated DTOs, repositories, services, dependency injection, database context, configuration, and seed data to use ProductCategory. Cleaned up all references to the old Category entity, improving separation of concerns and enabling more flexible category management.
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Categories" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="ProductCategories" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Brands" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Branches" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Products" sheetId="4" state="visible" r:id="rId6"/>
@@ -2358,7 +2358,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="51.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7107,7 +7107,7 @@
       <c r="B22" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>398</v>
       </c>
       <c r="D22" s="1" t="n">

</xml_diff>

<commit_message>
Add IngredientCategory entity and related mappings
- Introduced IngredientCategory entity and EF Core configuration
- Registered IngredientCategories DbSet in RestaurantDbContext
- Set up foreign key from Ingredient to IngredientCategory (Restrict)
- Added data import record, AutoMapper profile, and seeder
- Updated RestaurantData.xlsx with new category data
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="ProductCategories" sheetId="1" state="visible" r:id="rId3"/>
@@ -17,6 +17,7 @@
     <sheet name="Images" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="ProductImages" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Units" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="IngredientCategories" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1176" uniqueCount="455">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -1279,6 +1280,120 @@
   </si>
   <si>
     <t xml:space="preserve">half-dz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh and frozen meats used for preparing restaurant dishes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poultry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chicken, duck, turkey, and other poultry products used in food preparation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fish, shrimp, crab, squid, clams, and other seafood ingredients.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vegetables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh vegetables used in cooking, salads, soups, and side dishes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fruits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh and processed fruits used in dishes, desserts, beverages, and garnishes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Herbs &amp; Spices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh herbs, dried herbs, spices, and seasonings used to enhance flavor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grains &amp; Cereals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rice, wheat, oats, corn, and other grain-based ingredients.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noodles &amp; Pasta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rice noodles, wheat noodles, pasta, and other noodle products.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dairy &amp; Eggs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Milk, cheese, butter, cream, yogurt, eggs, and other dairy products.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sauces &amp; Condiments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soy sauce, fish sauce, ketchup, mayonnaise, chili sauce, and other condiments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oils &amp; Fats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cooking oils, shortening, lard, and other fats used for cooking and frying.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baking Ingredients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flour, baking powder, sugar, yeast, cocoa powder, and other baking ingredients.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuts &amp; Seeds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peanuts, almonds, sesame, cashews, and other nuts and seeds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legumes &amp; Beans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soybeans, tofu, chickpeas, lentils, beans, and other legume-based ingredients.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frozen Foods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frozen vegetables, seafood, meat, and other ingredients stored in frozen condition.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canned &amp; Preserved Foods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canned, pickled, dried, fermented, and otherwise preserved food ingredients.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingredients and beverage products used for preparing or serving drinks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweeteners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sugar, honey, syrup, artificial sweeteners, and other sweetening ingredients.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bakery &amp; Bread</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bread, buns, rolls, and other bakery products used as ingredients or side items.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepared Ingredients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-prepared ingredients such as stock, broth, spice mixes, and ready-to-use food components.</t>
   </si>
 </sst>
 </file>
@@ -1371,7 +1486,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1401,6 +1516,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1779,6 +1898,197 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="77.31"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>417</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>428</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
+        <v>436</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>438</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>440</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>442</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>446</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>449</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>454</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
Add IngredientStock entity, seeding, and mapping support
- Introduced IngredientStock entity with partial methods for IDs
- Registered IngredientStocks in RestaurantDbContext and model config
- Added IngredientStockSeeder for importing and linking stock data
- Created IngredientStockRecord DTO and AutoMapper profile
- Updated DatabaseSeeder to include IngredientStockSeeder
- Modified RestaurantData.xlsx to include stock data
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="11"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="ProductCategories" sheetId="1" state="visible" r:id="rId3"/>
@@ -20,6 +20,7 @@
     <sheet name="IngredientCategories" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="Ingredients" sheetId="11" state="visible" r:id="rId13"/>
     <sheet name="IngredientPrices" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="IngredientStocks" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1580" uniqueCount="612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1727" uniqueCount="612">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -4281,6 +4282,831 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C73"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.77"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>64</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>59</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>92</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>62</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>96</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>60</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="n">
+        <v>98</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="n">
+        <v>72</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="n">
+        <v>71</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="n">
+        <v>91</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="n">
+        <v>90</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="n">
+        <v>60</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="n">
+        <v>88</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="n">
+        <v>57</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="n">
+        <v>67</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="n">
+        <v>92</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="n">
+        <v>52</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="n">
+        <v>96</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0" t="n">
+        <v>88</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="n">
+        <v>58</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="n">
+        <v>75</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="n">
+        <v>63</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="n">
+        <v>68</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="n">
+        <v>97</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="n">
+        <v>70</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>587</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="n">
+        <v>56</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="0" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0" t="n">
+        <v>98</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="n">
+        <v>90</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>607</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>609</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
Add authentication with JWT and user/role services
Introduced authentication functionality with JWT token generation. Added interfaces and implementations for user and role repositories, authentication service, and related DTOs. Updated dependency injection to register new services for secure user login.
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="15"/>
   </bookViews>
   <sheets>
     <sheet name="ProductCategories" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,6 +23,7 @@
     <sheet name="IngredientStocks" sheetId="13" state="visible" r:id="rId15"/>
     <sheet name="Recipes" sheetId="14" state="visible" r:id="rId16"/>
     <sheet name="RecipeIngredients" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="Roles" sheetId="16" state="visible" r:id="rId18"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2968" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2986" uniqueCount="678">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -2017,6 +2018,57 @@
   </si>
   <si>
     <t xml:space="preserve">Sauté mushrooms, pumpkin and onion in butter, simmer with stock, blend until smooth, finish with cream, and season.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuperAdmin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Has full access to all system features and administrative functions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages restaurant operations, users, branches, products, inventory, and system settings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages daily operations of assigned restaurant branches, including employees, inventory, orders, and reports.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handles customer payments, invoices, orders, and checkout operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages food preparation, recipes, ingredients, and kitchen-related operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InventoryManager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages ingredients, stock levels, stock movements, suppliers, and inventory operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handles customer orders, tables, and order-related operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can browse products, place orders, manage their profile, and make payments.</t>
   </si>
 </sst>
 </file>
@@ -2028,7 +2080,7 @@
     <numFmt numFmtId="165" formatCode="h:mm"/>
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2056,6 +2108,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -2101,7 +2161,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2136,6 +2196,14 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -11021,6 +11089,100 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="88.09"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>661</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>662</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
+        <v>664</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
+        <v>666</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>670</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>672</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>674</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>677</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -13810,7 +13972,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="94.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="94.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add RoleSeeder and related mapping for role data seeding
Added RoleSeeder to seed roles from external data. Introduced RoleRecord and RoleMapping for data mapping. Updated DatabaseSeeder to include RoleSeeder. Registered required namespaces and dependencies. Updated RestaurantData.xlsx to support new role data.
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2986" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2986" uniqueCount="677">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -2018,9 +2018,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sauté mushrooms, pumpkin and onion in butter, simmer with stock, blend until smooth, finish with cream, and season.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Role Name</t>
   </si>
   <si>
     <t xml:space="preserve">SuperAdmin</t>
@@ -11097,12 +11094,13 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="88.09"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>661</v>
+        <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>1</v>
@@ -11110,66 +11108,66 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
+        <v>661</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>662</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
+        <v>663</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>664</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
+        <v>665</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>666</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
+        <v>667</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>668</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
+        <v>669</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>670</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>671</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
+        <v>671</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>672</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>673</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
+        <v>673</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>674</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
+        <v>675</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>676</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>677</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add StockStatus enum and update DTOs with status
Introduce StockStatus enum and StockStatusExtensions for inventory status logic. Update IngredientStockResponse and ProductStockResponse DTOs to include Status property. Adjust AutoMapper profiles to map Status using extension method. Restrict CustomersController authorization to "Customer" role only. Add necessary usings.
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="15"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="ProductCategories" sheetId="1" state="visible" r:id="rId3"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2986" uniqueCount="677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3146" uniqueCount="677">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -2158,7 +2158,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2195,12 +2195,8 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -11094,8 +11090,8 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="88.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="88.09"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11107,66 +11103,66 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="2" t="s">
         <v>661</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="2" t="s">
         <v>662</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="2" t="s">
         <v>663</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="2" t="s">
         <v>664</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="2" t="s">
         <v>665</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="2" t="s">
         <v>666</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="2" t="s">
         <v>667</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="2" t="s">
         <v>668</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="2" t="s">
         <v>669</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="2" t="s">
         <v>670</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="2" t="s">
         <v>671</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="2" t="s">
         <v>672</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="2" t="s">
         <v>673</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="2" t="s">
         <v>674</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="2" t="s">
         <v>675</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="2" t="s">
         <v>676</v>
       </c>
     </row>
@@ -13711,7 +13707,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
@@ -13948,6 +13944,886 @@
       </c>
       <c r="C21" s="3" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add personnel management domain with new entities
Introduced Department, Position, and Employee entities with relationships and EmployeeStatus enum. Updated User entity for one-to-one Employee link. Added EF Core configurations and sequence for Employee codes. Modified RestaurantDbContext and updated seed data.
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="ProductCategories" sheetId="1" state="visible" r:id="rId3"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3146" uniqueCount="677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3722" uniqueCount="677">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -4497,7 +4497,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C361"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.76"/>
@@ -5304,6 +5304,3174 @@
       </c>
       <c r="C73" s="3" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="1" t="n">
+        <v>97</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B147" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B150" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C150" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="C151" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="C153" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="C154" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="C155" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="C156" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="C157" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B158" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="C159" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B160" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="C161" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="C162" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="C163" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B164" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C164" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B165" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="C165" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="C166" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="C167" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="C168" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="C169" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="C170" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B171" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="C171" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B172" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="C172" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="C173" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B174" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="C174" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B175" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="C175" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B176" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="C176" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="C177" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="C178" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B179" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="C179" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B180" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B181" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="C181" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B182" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="C182" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B183" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C183" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B184" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="C184" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="185" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B185" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="C185" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="186" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="C186" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B187" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="C187" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B188" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="C188" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B189" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="C189" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="190" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B190" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="C190" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="191" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B191" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="C191" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B192" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="C192" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A193" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B193" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="C193" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="194" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="B194" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="C194" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A195" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B195" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="C195" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="196" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A196" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B196" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="C196" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B197" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="C197" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B198" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="C198" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B199" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="C199" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B200" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="C200" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B201" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="C201" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B202" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="C202" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="203" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B203" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="C203" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B204" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="C204" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="1" t="n">
+        <v>97</v>
+      </c>
+      <c r="B205" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="C205" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="206" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B206" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="C206" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B207" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="C207" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A208" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B208" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A209" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B209" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="C209" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="210" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A210" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B210" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="C210" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="211" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A211" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B211" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C211" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B212" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B213" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="C213" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B214" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="C214" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B215" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="C215" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B216" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="C216" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B217" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="C217" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B218" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="C218" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B219" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="C219" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B220" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="C220" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B221" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C221" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B222" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C222" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B223" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="C223" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B224" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="C224" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B225" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B226" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="C226" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="C227" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="B228" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B229" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="C229" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B230" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B231" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B232" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B233" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="234" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B234" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="C234" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B235" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B236" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C236" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="C237" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="238" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="C238" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="C239" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="240" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B240" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="241" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B241" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="C241" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="242" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="C242" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="243" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="C243" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="244" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="C244" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="245" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="C245" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="246" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="C246" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="247" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="C247" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="248" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="249" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="C249" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="250" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A250" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="C250" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="251" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A251" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="C251" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="252" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A252" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="253" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A253" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="C253" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="254" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A254" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="255" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A255" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C255" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="256" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A256" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="257" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A257" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="C257" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="258" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="C258" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="259" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="C259" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="260" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="261" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="C261" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="262" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="263" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A263" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B263" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="C263" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="264" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B264" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="265" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A265" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="C265" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="266" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="C266" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="267" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A267" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="C267" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="268" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A268" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="C268" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="269" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A269" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B269" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="C269" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="270" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A270" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B270" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="C270" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="271" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A271" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="C271" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="272" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A272" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B272" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="273" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A273" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B273" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="C273" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="274" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A274" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="C274" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="275" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A275" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="C275" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="276" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A276" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B276" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="C276" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="277" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A277" s="1" t="n">
+        <v>97</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="C277" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="278" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A278" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="C278" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="279" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A279" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B279" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="C279" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="280" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A280" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C280" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="281" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A281" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="C281" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="282" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A282" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B282" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="C282" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="283" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A283" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C283" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="284" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A284" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="C284" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="285" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A285" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="C285" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="286" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A286" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="C286" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="287" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A287" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="C287" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="288" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A288" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="C288" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="289" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A289" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B289" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="C289" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="290" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A290" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="C290" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="291" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A291" s="1" t="n">
+        <v>59</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="C291" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="292" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A292" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="C292" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="293" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A293" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C293" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="294" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A294" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C294" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="295" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A295" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="C295" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="296" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A296" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="C296" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="297" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A297" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="C297" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="298" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A298" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B298" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="C298" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="299" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A299" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B299" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="C299" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="300" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A300" s="1" t="n">
+        <v>99</v>
+      </c>
+      <c r="B300" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="C300" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="301" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A301" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="C301" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="302" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A302" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="C302" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="303" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A303" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B303" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="C303" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="304" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A304" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="C304" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="305" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A305" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="C305" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="306" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A306" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="C306" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="307" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A307" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="C307" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="308" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A308" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C308" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="309" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A309" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="C309" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="310" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A310" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="C310" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="311" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A311" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B311" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="C311" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="312" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A312" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="B312" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="C312" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="313" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A313" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B313" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="C313" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="314" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A314" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B314" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="C314" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="315" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A315" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="C315" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="316" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A316" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="C316" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="317" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A317" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B317" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="C317" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="318" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A318" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B318" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="C318" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="319" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A319" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="B319" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="C319" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="320" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A320" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B320" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="C320" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="321" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A321" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B321" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="C321" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="322" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A322" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B322" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="C322" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="323" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A323" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B323" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="C323" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="324" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A324" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B324" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C324" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="325" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A325" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B325" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="C325" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="326" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A326" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B326" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="C326" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="327" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A327" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B327" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C327" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="328" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A328" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B328" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="C328" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="329" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A329" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B329" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="C329" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="330" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A330" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B330" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="C330" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="331" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A331" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B331" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="C331" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="332" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A332" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B332" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="C332" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="333" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A333" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B333" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="C333" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="334" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A334" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="C334" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="335" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A335" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="C335" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="336" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A336" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="C336" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="337" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A337" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B337" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="C337" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="338" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A338" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="C338" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="339" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A339" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="C339" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="340" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A340" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B340" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="C340" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="341" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A341" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B341" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="C341" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="342" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A342" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B342" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="C342" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="343" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A343" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B343" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="C343" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="344" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A344" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B344" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="C344" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="345" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A345" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B345" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="C345" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="346" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A346" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B346" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="C346" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="347" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A347" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B347" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="C347" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="348" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A348" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B348" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="C348" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="349" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A349" s="1" t="n">
+        <v>97</v>
+      </c>
+      <c r="B349" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="C349" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="350" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A350" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B350" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="C350" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="351" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A351" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B351" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="C351" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="352" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A352" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B352" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C352" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="353" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A353" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B353" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="C353" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="354" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A354" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="C354" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="355" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A355" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B355" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C355" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="356" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A356" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B356" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="C356" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="357" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A357" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B357" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="C357" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="358" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A358" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B358" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="C358" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="359" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A359" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B359" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="C359" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="360" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A360" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B360" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="C360" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="361" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A361" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B361" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="C361" s="3" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add seeding for Department and Position entities
Introduce Department/Position seeders, mapping profiles, and data records. Update DbContext and DatabaseSeeder. Refactor Position entity and update RestaurantData.xlsx.
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="ProductCategories" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,6 +24,8 @@
     <sheet name="Recipes" sheetId="14" state="visible" r:id="rId16"/>
     <sheet name="RecipeIngredients" sheetId="15" state="visible" r:id="rId17"/>
     <sheet name="Roles" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="Departments" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="Positions" sheetId="18" state="visible" r:id="rId20"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3722" uniqueCount="677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3835" uniqueCount="754">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -2066,6 +2068,237 @@
   </si>
   <si>
     <t xml:space="preserve">Can browse products, place orders, manage their profile, and make payments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees the overall business operations, performance, and administration of the restaurant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Front of House</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handles customer service, table service, guest reception, and other activities in the dining area.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kitchen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsible for food preparation, cooking, kitchen operations, and food quality.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar &amp; Beverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsible for preparing, serving, and managing beverages.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warehouse &amp; Inventory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages inventory, stock levels, storage, receiving, and issuing of ingredients and supplies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchasing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handles procurement of ingredients, supplies, equipment, and relationships with suppliers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finance &amp; Accounting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages financial transactions, revenue, expenses, invoices, payments, and accounting activities.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human Resources</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages employee records, recruitment, attendance, workforce administration, and HR policies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Information Technology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages the restaurant's IT infrastructure, software systems, website, and technical operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DepartmentName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees the overall operation and performance of the restaurant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assistant Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assists the General Manager in managing daily restaurant operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages the daily operations and performance of a specific restaurant branch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host / Hostess</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welcomes guests, manages seating arrangements, and assists with reservations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiter / Waitress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Takes customer orders, serves food and beverages, and assists guests during their dining experience.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handles customer payments, receipts, and related cashier operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receptionist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welcomes guests, handles reservations, and assists customers at the reception area.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shift Supervisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervises front-of-house employees and operations during an assigned shift.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Executive Chef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees kitchen operations, food quality, menu standards, and kitchen staff.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sous Chef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assists the Executive Chef and supervises daily kitchen operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepares and cooks dishes according to the restaurant's recipes and quality standards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kitchen Assistant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assists with ingredient preparation, kitchen equipment, and general kitchen tasks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dishwasher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cleans dishes, kitchen utensils, and maintains cleanliness in designated areas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees bar operations, beverage quality, inventory, and bar staff.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bartender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepares and serves beverages according to restaurant standards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar Assistant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assists with beverage preparation, ingredient preparation, equipment, and bar cleanliness.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warehouse Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees warehouse operations, storage, stock control, and inventory management.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inventory Controller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitors stock levels, inventory movements, and performs inventory checks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storekeeper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receives, stores, maintains, and issues ingredients and supplies from the warehouse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchasing Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees procurement activities and manages supplier relationships.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchasing Officer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Processes purchase orders, communicates with suppliers, and tracks procurement activities.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finance Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees financial operations, budgeting, financial control, and cash flow.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accountant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handles accounting records, invoices, revenue, expenses, and financial transactions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financial Controller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviews and controls financial transactions, reports, and accounting activities.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees human resource operations, employee management, recruitment, and HR policies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR Officer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handles employee records, recruitment support, attendance, and daily HR administration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oversees the restaurant's IT systems, infrastructure, and technical operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System Administrator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages servers, user accounts, system access, network infrastructure, and IT security.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web Administrator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manages website configuration, content, access, and day-to-day website operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software Developer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Develops, maintains, and improves the restaurant's website, APIs, and software systems.</t>
   </si>
 </sst>
 </file>
@@ -2158,7 +2391,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2197,6 +2430,14 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -14345,6 +14586,473 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.4"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
+        <v>677</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>681</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>683</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>687</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>689</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>691</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>693</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>694</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C31"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="79.74"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="10" t="s">
+        <v>695</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
+        <v>677</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>696</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="11" t="s">
+        <v>677</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>698</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>677</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>700</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>702</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>704</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>667</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>707</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>709</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="s">
+        <v>681</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>711</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>681</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>713</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
+        <v>681</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>681</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>716</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>681</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>718</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>683</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>720</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>683</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>722</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>683</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>724</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>726</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>728</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>730</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
+        <v>687</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>732</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>687</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>734</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>689</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>736</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
+        <v>689</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>738</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>689</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>740</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>691</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>742</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11" t="s">
+        <v>691</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>744</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
+        <v>693</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>746</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
+        <v>693</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>748</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>693</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>750</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
+        <v>693</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>752</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>753</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>